<commit_message>
update select com and uart log
</commit_message>
<xml_diff>
--- a/Image2Gcode/excel/time_processing.xlsx
+++ b/Image2Gcode/excel/time_processing.xlsx
@@ -128,6 +128,61 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>3</col>
+      <colOff>0</colOff>
+      <row>1</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="952500" cy="714375"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -417,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -454,18 +509,34 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
+    <row r="2" ht="85" customHeight="1">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1.jpg</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr"/>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>TỔNG: 0.000 giây</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1.598</v>
       </c>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>TỔNG: 1.598 giây</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
merging source code, add after finish draw rectangle
</commit_message>
<xml_diff>
--- a/Image2Gcode/excel/time_processing.xlsx
+++ b/Image2Gcode/excel/time_processing.xlsx
@@ -512,16 +512,16 @@
     <row r="2" ht="85" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1.jpg</t>
+          <t>4.jpg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="n">
-        <v>1.598</v>
+        <v>2.238</v>
       </c>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="n">
-        <v>401</v>
+        <v>481</v>
       </c>
     </row>
     <row r="3">
@@ -529,7 +529,7 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>TỔNG: 1.598 giây</t>
+          <t>TỔNG: 2.238 giây</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>

</xml_diff>